<commit_message>
README.me Q2 updated by THEO
</commit_message>
<xml_diff>
--- a/MCMC-ABC_results/resultats_complets.xlsx
+++ b/MCMC-ABC_results/resultats_complets.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Config" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Scan_delta" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Scaling_NITER" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scaling_NCHAINS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Baseline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scan_epsilon" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Scan_delta" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Scaling_NITER" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Scaling_NCHAINS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -813,7 +815,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -828,7 +830,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>8000</v>
+        <v>3000</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -843,7 +845,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>40000</v>
+        <v>15000</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
@@ -858,7 +860,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
@@ -873,7 +875,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -888,7 +890,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
@@ -903,7 +905,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -918,7 +920,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
@@ -940,7 +942,1908 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Baseline — ε=1  N_DATASETS=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>(A)=std posterior  (B)=std MC  (C)=std inter-datasets</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Métrique</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Formule / calcul</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Valeur (moy. datasets)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Std inter-datasets (C)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Interprétation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Biais μ</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>médiane_post − 0.0</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>-0.08001999999999999</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.00251</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>0 = pas de biais ABC. Diminue avec ε↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Biais σ</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>médiane_post − 0.3</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0.18157</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.00354</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0 = pas de biais ABC. Diminue avec ε↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Std posterior μ (A)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>std(160k échantillons poolés)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0.06561</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.00123</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Largeur de p(μ|Y). Propriété du modèle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Std posterior σ (A)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>std(160k échantillons poolés)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.09717000000000001</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.00325</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Largeur de p(σ|Y). Propriété du modèle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Std MC μ (B)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>std des 8 médianes inter-chaînes</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0.00295</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0.00128</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Stabilité estimateur. Diminue avec N_ITER↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Std MC σ (B)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>std des 8 médianes inter-chaînes</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.00725</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.00263</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Stabilité estimateur. Diminue avec N_ITER↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Largeur IC95 μ</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>q97.5 − q2.5 poolés</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.23842</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.00391</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Diminue avec ε↓ et M_OBS↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Largeur IC95 σ</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>q97.5 − q2.5 poolés</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0.35978</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.01194</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Diminue avec ε↓ et M_OBS↑</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>R-hat μ</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Gelman-Rubin (cible &lt; 1.01)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1.00066</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.00036</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Convergence inter-chaînes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>R-hat σ</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Gelman-Rubin (cible &lt; 1.01)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>1.00219</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.00116</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Convergence inter-chaînes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>ESS ratio μ</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>ESS / (N_CHAINS × N_ITER)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0.01079</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Efficacité mixing. 1.0=parfait</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ESS ratio σ</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>ESS / (N_CHAINS × N_ITER)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0.00582</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.0009300000000000001</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Efficacité mixing. 1.0=parfait</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Acceptance rate</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>moy. sur 8 chaînes</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>0.15615</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.00124</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Cible 20–40%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Scan ε — 30 valeurs  N_DATASETS=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Chaque ligne = une valeur de ε. Colonnes _mean/_std_ds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>epsilon</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>bias_mu_mean</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>bias_mu_std_ds</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>bias_sigma_mean</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>bias_sigma_std_ds</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>acc_mean_mean</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>acc_mean_std_ds</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>ess_ratio_mu_mean</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>ess_ratio_mu_std_ds</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>ic95_width_mu_mean</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>ic95_width_mu_std_ds</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>rhat_mu_mean</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>rhat_mu_std_ds</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>std_mc_mu_mean</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>std_mc_mu_std_ds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>-0.02963</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>0.05237</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.10727</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.17519</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0.00054</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0.16688</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.14396</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.06109</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.09470000000000001</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>1.33378</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0.49091</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>0.02783</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>0.046</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>0.15172</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>-0.00563</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0.00693</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.01825</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>0.01397</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.01246</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0.00134</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0.0006400000000000001</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>0.06414</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0.03768</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>1.08503</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0.14083</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0.01691</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>0.02737</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>0.25345</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>-0.00937</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0.00323</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.02939</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0.00637</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0.02866</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0.00397</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.00344</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.00081</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0.08476</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0.02854</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>1.08021</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0.13863</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0.00487</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>0.00652</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>0.35517</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>-0.0151</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0.00162</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.04806</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.00534</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.04735</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.00322</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0.00348</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0.00034</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>0.09152</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0.00283</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>1.00092</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0.00043</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0.00119</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>9.000000000000001e-05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>0.4569</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>-0.02527</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0.00092</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0.07072000000000001</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0.00614</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.06517000000000001</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>0.00123</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0.00464</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.00018</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0.11404</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0.00285</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>1.00329</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0.00203</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>0.00267</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>0.00103</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>0.55862</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>-0.03492</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0.00103</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.09314</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.00424</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.08026999999999999</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.00114</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0.00561</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0.00028</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>0.13593</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0.00273</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>1.0021</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>0.00219</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0.00258</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>0.66034</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>-0.04414</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.00218</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.11445</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0.00511</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0.09775</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0.00176</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0.00694</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.00124</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0.15786</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0.00522</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>1.00048</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0.00021</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0.00184</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>0.00095</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>0.76207</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>-0.05423</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0.00086</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.13514</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.00355</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.11351</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0.00856</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0.00161</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>0.18164</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.00495</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>1.00092</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>0.00146</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>0.8637899999999999</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>-0.06401</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0.00212</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.1546</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0.00615</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.13225</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0.00349</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0.00778</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.00235</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0.20491</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>1.00065</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0.00049</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0.00245</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>0.00046</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>0.96552</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>-0.07568</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0.00136</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.17419</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.00502</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.14872</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.00266</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0.00919</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0.00048</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>0.22965</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>0.0009300000000000001</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>1.00079</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0.00067</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0.00359</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>0.00164</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>1.06724</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>-0.08581999999999999</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0.00017</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.19254</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.00558</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.1675</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0.00329</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0.01151</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.00113</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0.25263</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0.00301</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>1.00099</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0.00074</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0.00436</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>0.00126</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>1.16897</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>-0.09702</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0.00125</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.21069</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.00546</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.18281</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.00211</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0.01085</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0.00281</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>0.28134</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0.00414</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>1.00042</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0.00018</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0.00321</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>1.27069</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>-0.10836</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>0.00237</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.22834</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>8.000000000000001e-05</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.202</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0.00086</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0.01159</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.00137</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0.30569</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>0.00256</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>1.0008</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>0.00037</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>0.00368</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0.00029</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>1.37241</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>-0.11737</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0.00276</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0.24129</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0.00297</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.22067</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0.00194</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>0.01288</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>0.00342</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>0.33427</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>0.00241</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>1.00033</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>0.00022</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>0.00312</v>
+      </c>
+      <c r="O17" s="5" t="n">
+        <v>0.00125</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>1.47414</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>-0.12768</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0.00512</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0.25578</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0.00408</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.23616</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0.00245</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0.01359</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.00236</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0.36037</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>0.00063</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>1.00035</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0.00022</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>0.00418</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>0.00032</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>1.57586</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>-0.13993</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0.00079</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0.27214</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0.00357</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.25312</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0.00401</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0.01384</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>0.38967</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>0.00101</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>1.00052</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>0.00039</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>0.00398</v>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>0.00136</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>1.67759</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>-0.14947</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0.00083</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0.28551</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0.00299</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0.27029</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0.00138</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0.01494</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.00233</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0.41566</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>0.00495</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>1.00041</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0.00047</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>0.00354</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>0.00189</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>1.77931</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>-0.15857</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0.00388</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0.29971</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.00161</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0.2866</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0.00107</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0.01496</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>0.00198</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>0.4414</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>0.00632</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>1.0005</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="N21" s="5" t="n">
+        <v>0.0049</v>
+      </c>
+      <c r="O21" s="5" t="n">
+        <v>0.00137</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>1.88103</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>-0.16894</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0.00152</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.31138</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0.30191</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0.00235</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0.0146</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.00079</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0.46936</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>0.00306</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>1.00066</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>0.00051</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>0.00523</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>0.00156</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>1.98276</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>-0.18294</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>0.00349</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0.3273</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0.00473</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0.31914</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0.00154</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>0.01487</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>9.000000000000001e-05</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>0.00117</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>1.00062</v>
+      </c>
+      <c r="M23" s="5" t="n">
+        <v>0.00037</v>
+      </c>
+      <c r="N23" s="5" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="O23" s="5" t="n">
+        <v>0.00239</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>2.08448</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>-0.19259</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0.00211</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0.33783</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0.0083</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0.33441</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0.00304</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0.01486</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0.52557</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0.00273</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>1.00004</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>6e-05</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>0.00248</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>0.00012</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>2.18621</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>-0.2003</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>0.00311</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0.34761</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0.00728</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0.34872</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0.00091</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>0.01594</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>0.00182</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>0.55791</v>
+      </c>
+      <c r="K25" s="5" t="n">
+        <v>0.00129</v>
+      </c>
+      <c r="L25" s="5" t="n">
+        <v>1.00058</v>
+      </c>
+      <c r="M25" s="5" t="n">
+        <v>0.00036</v>
+      </c>
+      <c r="N25" s="5" t="n">
+        <v>0.00677</v>
+      </c>
+      <c r="O25" s="5" t="n">
+        <v>0.00086</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>2.28793</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>-0.21203</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0.00321</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0.35851</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0.00212</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.36433</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0.00166</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0.01498</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0.00139</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>0.58657</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0.00598</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>1.00033</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>0.00013</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>0.00494</v>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>0.00062</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>2.38966</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>-0.2165</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>0.00341</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>0.36396</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>0.00678</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0.37954</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0.00211</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>0.01561</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>0.6158400000000001</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>0.00223</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>1.00084</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>0.00095</v>
+      </c>
+      <c r="N27" s="5" t="n">
+        <v>0.00653</v>
+      </c>
+      <c r="O27" s="5" t="n">
+        <v>0.00418</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>2.49138</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>-0.23148</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0.00393</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0.37752</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0.00344</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.39433</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0.00135</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0.01559</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>0.64674</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>0.008670000000000001</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>1.00069</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>0.00041</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>0.00754</v>
+      </c>
+      <c r="O28" s="4" t="n">
+        <v>0.00223</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>2.5931</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>-0.24138</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>0.00447</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>0.39179</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>0.00477</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0.40651</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>0.00092</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>0.01365</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>0.00146</v>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>0.67462</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="L29" s="5" t="n">
+        <v>1.00061</v>
+      </c>
+      <c r="M29" s="5" t="n">
+        <v>0.00058</v>
+      </c>
+      <c r="N29" s="5" t="n">
+        <v>0.00698</v>
+      </c>
+      <c r="O29" s="5" t="n">
+        <v>0.00283</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>2.69483</v>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>-0.24778</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0.00308</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0.39762</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0.00087</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.42014</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0.00249</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0.01783</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0.00069</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>0.70853</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>0.00371</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>1.00045</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>0.00039</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="O30" s="4" t="n">
+        <v>0.00309</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>2.79655</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>-0.25856</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>0.00593</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>0.40449</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0.00568</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0.43242</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0.00157</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0.01599</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0.00046</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0.73111</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.00254</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>1.0006</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>0.00047</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>0.00796</v>
+      </c>
+      <c r="O31" s="5" t="n">
+        <v>0.00327</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>2.89828</v>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>-0.26733</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0.0067</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>0.41445</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.00777</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.44359</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0.00392</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>0.01573</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>0.00189</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>0.76534</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0.00272</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>1.00041</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>0.00023</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>0.00673</v>
+      </c>
+      <c r="O32" s="4" t="n">
+        <v>0.00212</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>-0.27722</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>0.00355</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>0.4225</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0.45271</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0.00291</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>0.01533</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>0.00189</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>0.79749</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>1.0004</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>0.00043</v>
+      </c>
+      <c r="N33" s="5" t="n">
+        <v>0.00728</v>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>0.00503</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -961,7 +2864,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Scan δ — 7 valeurs  ε=1.5 fixé</t>
+          <t>Scan δ — 30 valeurs  ε=1 fixé</t>
         </is>
       </c>
     </row>
@@ -1044,286 +2947,1229 @@
         <v>0.01</v>
       </c>
       <c r="B4" s="4" t="n">
-        <v>0.94942</v>
+        <v>0.89879</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>0.00168</v>
+        <v>0.00556</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.0007</v>
+        <v>0.00127</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3e-05</v>
+        <v>0.00028</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>-0.128</v>
+        <v>-0.08776</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.0053</v>
+        <v>0.00245</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.2595</v>
+        <v>0.19443</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>0.0165</v>
+        <v>0.00564</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1.01872</v>
+        <v>1.02431</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>0.01269</v>
+        <v>0.0128</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>0.02028</v>
+        <v>0.01447</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0.00753</v>
+        <v>0.00615</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>0.14167</v>
+        <v>0.03724</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.44099</v>
+        <v>0.74527</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.00139</v>
+        <v>0.00135</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.009140000000000001</v>
+        <v>0.00347</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.00051</v>
+        <v>0.00046</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.13211</v>
+        <v>-0.08232</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.00222</v>
+        <v>0.00248</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0.26329</v>
+        <v>0.18557</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>0.00444</v>
+        <v>0.00251</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>1.00032</v>
+        <v>1.00355</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>0.00029</v>
+        <v>0.00179</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>0.00262</v>
+        <v>0.00595</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>0.00112</v>
+        <v>0.00208</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>0.27333</v>
+        <v>0.06448</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>0.21463</v>
+        <v>0.59501</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0.00094</v>
+        <v>0.00134</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.01107</v>
+        <v>0.00496</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.00045</v>
+        <v>0.00059</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>-0.13217</v>
+        <v>-0.07982</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.0039</v>
+        <v>0.00251</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>0.26278</v>
+        <v>0.1806</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.00395</v>
+        <v>0.0075</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1.00027</v>
+        <v>1.00135</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>0.00018</v>
+        <v>0.00179</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>0.00338</v>
+        <v>0.00301</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>0.00092</v>
+        <v>0.0024</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>0.405</v>
+        <v>0.09172</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>0.12207</v>
+        <v>0.47213</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0.0008899999999999999</v>
+        <v>0.00208</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.008019999999999999</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.00036</v>
+        <v>0.00109</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0.13178</v>
+        <v>-0.07784000000000001</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.00241</v>
+        <v>0.00145</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>0.263</v>
+        <v>0.17891</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.00234</v>
+        <v>0.00301</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>1.00053</v>
+        <v>1.00063</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.0009</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>0.00418</v>
+        <v>0.00273</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>0.00102</v>
+        <v>0.00181</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>0.53667</v>
+        <v>0.11897</v>
       </c>
       <c r="B8" s="4" t="n">
-        <v>0.07746</v>
+        <v>0.37433</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0.00056</v>
+        <v>0.00139</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.00576</v>
+        <v>0.00992</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.00049</v>
+        <v>0.00126</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>-0.13095</v>
+        <v>-0.07954</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.00363</v>
+        <v>0.00159</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.26211</v>
+        <v>0.18251</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0036</v>
+        <v>0.00399</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1.00019</v>
+        <v>1.00072</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>0.00011</v>
+        <v>0.00019</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>0.00282</v>
+        <v>0.00311</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>0.00084</v>
+        <v>0.00077</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>0.66833</v>
+        <v>0.14621</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0.05261</v>
+        <v>0.30067</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.00039</v>
+        <v>0.00183</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.00439</v>
+        <v>0.01028</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.00032</v>
+        <v>0.00174</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.13074</v>
+        <v>-0.07811999999999999</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.00403</v>
+        <v>0.00306</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0.26253</v>
+        <v>0.17978</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0.00445</v>
+        <v>0.00147</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>1.0009</v>
+        <v>1.00037</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0.0003</v>
+        <v>0.00027</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0.00543</v>
+        <v>0.00298</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>0.00154</v>
+        <v>0.00082</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
+        <v>0.17345</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0.24984</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.00171</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.01076</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0.00077</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>-0.07889</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0.00211</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0.18122</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.00582</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>1.00048</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0.00032</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0.00263</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0.00135</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>0.20069</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0.2069</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0.00155</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.01172</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.00106</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>-0.07918</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.00304</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0.18191</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0.00359</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>1.00029</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.00014</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>0.00258</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0.00014</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>0.22793</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0.17505</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>6e-05</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.0086</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0.00091</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>-0.08014</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0.00184</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0.18156</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.00398</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>1.00038</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0.00028</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0.00264</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0.00073</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>0.25517</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0.14901</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0.00163</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.01034</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>-0.08198</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.00195</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0.18356</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0.00349</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>1.0006</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>0.00032</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>0.00357</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0.00165</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>0.28241</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.009650000000000001</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.00148</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>-0.07969999999999999</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0.00157</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0.18396</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.00466</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>1.00093</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0.00041</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0.00368</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0.00078</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>0.30966</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0.11133</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0.00242</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.008869999999999999</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.00149</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>-0.07862</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.00083</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0.18165</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0.00533</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>1.00121</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0.00085</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>0.00389</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0.00217</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>0.3369</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>0.10039</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>0.00161</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0.00023</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>-0.07882</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0.00259</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0.17931</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.00685</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>1.00064</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>0.00021</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>0.36414</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0.08645</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0.00713</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0.00046</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>-0.07914</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0.00161</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>0.18342</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>0.00766</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>1.00149</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>0.00079</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>0.00496</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>0.00281</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>0.39138</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>0.07713</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0.00024</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0.00564</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0.00127</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>-0.08198999999999999</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0.00128</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0.18556</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.01003</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>1.0022</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>0.00131</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0.00597</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0.00207</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>0.41862</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0.07106999999999999</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0.00038</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0.00647</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0.00054</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>-0.07675999999999999</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0.00197</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0.17794</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>0.00851</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>1.00368</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>0.00327</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>0.00515</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>0.00151</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>0.44586</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>0.06269</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0.00114</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0.00624</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0.00126</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>-0.07971</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0.17921</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.00569</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>1.00042</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>0.00044</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>0.00239</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0.00134</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>0.4731</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0.0575</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0.00106</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0.00545</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.00021</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>-0.07661</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0.00154</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0.17781</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>0.00443</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>1.00123</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>0.00113</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>0.0049</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>0.50034</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>0.05186</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.00466</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>-0.07819</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0.00242</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0.18158</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.00722</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>1.00136</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>0.00024</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>0.00422</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>0.00148</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>0.52759</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0.04647</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0.00498</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0.00088</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>-0.08132</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>0.18128</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>0.00238</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>1.00346</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>0.00218</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>0.0056</v>
+      </c>
+      <c r="M23" s="5" t="n">
+        <v>0.00232</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>0.55483</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>0.04311</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0.00039</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0.00406</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0.00045</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>-0.08033</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0.00102</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0.1839</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.00705</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>1.00086</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0.00111</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0.00378</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>0.0024</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>0.58207</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0.03867</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>0.00113</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0.00397</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0.00069</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>-0.08074000000000001</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0.00221</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>0.18282</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>0.00546</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>1.00251</v>
+      </c>
+      <c r="K25" s="5" t="n">
+        <v>0.00176</v>
+      </c>
+      <c r="L25" s="5" t="n">
+        <v>0.00631</v>
+      </c>
+      <c r="M25" s="5" t="n">
+        <v>0.00222</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>0.60931</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>0.03627</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>0.00077</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0.00363</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0.0009300000000000001</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>-0.08230999999999999</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0.18513</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0.00783</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>1.00358</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0.00159</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0.00461</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>0.0025</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>0.6365499999999999</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0.03346</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>0.00376</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>0.00024</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>-0.07883999999999999</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0.00083</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>0.18204</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>0.008710000000000001</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>1.00228</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>0.00072</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>0.00469</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>0.00099</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>0.66379</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>0.03139</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0.00267</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0.00022</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>-0.07875</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0.17562</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0.00686</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>1.00275</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>0.00234</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>0.00701</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>0.00256</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>0.69103</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0.02888</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>0.00021</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>0.00267</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>0.00022</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>-0.07685</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>0.00296</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>0.18176</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>0.00683</v>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>1.00182</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>0.00094</v>
+      </c>
+      <c r="L29" s="5" t="n">
+        <v>0.00587</v>
+      </c>
+      <c r="M29" s="5" t="n">
+        <v>0.00255</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>0.71828</v>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>0.02663</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0.00024</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0.00283</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0.00053</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0.00642</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0.17574</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0.00644</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>1.00337</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>0.00766</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>0.0034</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>0.74552</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0.02508</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>0.00038</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>0.00276</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0.00053</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>-0.07831</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0.00838</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0.1789</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0.00542</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>1.00162</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.00116</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>0.00507</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>0.00302</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>0.77276</v>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>0.02354</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0.00027</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>0.00272</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.00045</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>-0.07606</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0.00403</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>0.17974</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>0.00345</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>1.00204</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0.00188</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>0.00684</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>0.00348</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>0.03788</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>0.00028</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0.00309</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>0.00049</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>-0.1314</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>0.0045</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>0.26155</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>0.00186</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>1.00058</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>0.00034</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>0.00474</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>0.0014</v>
+      <c r="B33" s="5" t="n">
+        <v>0.02212</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>0.00035</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>0.00276</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>-0.08044</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0.00371</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>0.17697</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>1.00763</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>0.00655</v>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>0.01086</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>0.0029</v>
       </c>
     </row>
   </sheetData>
@@ -1335,17 +4181,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1372,55 +4218,119 @@
         <v>500</v>
       </c>
       <c r="B3" s="4" t="n">
-        <v>297.3198</v>
+        <v>7.2065</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>4583</v>
+        <v>2250</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>432.691</v>
+        <v>9.850199999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>8667</v>
+        <v>4000</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>571.3817</v>
+        <v>12.2557</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>12750</v>
+        <v>5750</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>726.1562</v>
+        <v>14.192</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>16833</v>
+        <v>7500</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>849.9031</v>
+        <v>18.9185</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>20917</v>
+        <v>9250</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1010.0939</v>
+        <v>22.5711</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
+        <v>11000</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>22.075</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>12750</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>24.5245</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>14500</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>27.4444</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>16250</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>31.2679</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>18000</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>33.3026</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>19750</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>34.8591</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>21500</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>37.5656</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>23250</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>41.1774</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
         <v>25000</v>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>1133.8647</v>
+      <c r="B17" s="4" t="n">
+        <v>45.8202</v>
       </c>
     </row>
   </sheetData>
@@ -1431,17 +4341,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1468,7 +4378,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="n">
-        <v>347.0515</v>
+        <v>10.45</v>
       </c>
     </row>
     <row r="4">
@@ -1476,7 +4386,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>645.0051</v>
+        <v>16.3249</v>
       </c>
     </row>
     <row r="5">
@@ -1484,7 +4394,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1036.4082</v>
+        <v>23.1316</v>
       </c>
     </row>
     <row r="6">
@@ -1492,7 +4402,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1269.6461</v>
+        <v>27.7813</v>
       </c>
     </row>
     <row r="7">
@@ -1500,7 +4410,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>1652.7087</v>
+        <v>36.2746</v>
       </c>
     </row>
     <row r="8">
@@ -1508,7 +4418,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1985.9562</v>
+        <v>41.9101</v>
       </c>
     </row>
     <row r="9">
@@ -1516,7 +4426,79 @@
         <v>7</v>
       </c>
       <c r="B9" s="4" t="n">
-        <v>2347.4937</v>
+        <v>48.2476</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>53.4632</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>66.0317</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>75.3347</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>80.52809999999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>86.16759999999999</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>89.5307</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>92.3152</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>99.12569999999999</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>105.802</v>
       </c>
     </row>
   </sheetData>

</xml_diff>